<commit_message>
feat(balance): L01 血量五轮调优，W15-25 地面累计约 ×3.73
沿 hp-20261030 链做五轮增量：W5-25 地面 ×1.25 / 空中 ×1.05 → 地面再 ×1.55 / 空中 ×1.05 → W10-25 地面 ×0.85 → W15-25 地面 ×0.9 → W15-25 地面 ×0.95。最终相对初版：地面 W5-9 ×4.359、W10-14 约 ×3.705、W15-25 约 ×3.727；空中 ×4.41；W1-4、数量、奖励、出怪间隔、三塔与 par 不动，expectedEnemyCount 仍 10236。

- Levels/L01/EnemyData.xlsx：100 个 W5-25 变体 hp 与 desc 标注；EnemyList.xlsx 同步各波 EHP 描述。
- 30 关 LevelRating 重封 runtimeContentHash=cc53b074…（9 键版 reseal），L01 planHash 与 balanceRevision=hp5-ground95-20261030-v1 更新。
- ConfigJson 的 tbenemydata / tbenemylist / tblevelrating 同步为导出产物。
- 证据 Docs/BalanceEvidence/L01-HP-Tune-20261030/：README 五段与 6 个调优脚本，每个脚本的护栏都要求基线是上一轮状态。

验证：Luban 导出 ×2 → Play Mode [Rating] verified cc53b074…，0 error → 运行时抽查 W15 普通怪 hp=208.1944。README 中"配合失败续局游玩"一句属当时语境，续局链路已于同日删除。
</commit_message>
<xml_diff>
--- a/Luban/Config/Datas/Levels/L01/EnemyData.xlsx
+++ b/Luban/Config/Datas/Levels/L01/EnemyData.xlsx
@@ -1731,7 +1731,7 @@
         <v>1.106615</v>
       </c>
       <c r="D10" s="0" t="n">
-        <v>39.538654</v>
+        <v>76.606143</v>
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
@@ -1770,7 +1770,7 @@
       <c r="O10" s="0" t="n"/>
       <c r="P10" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=5 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=5 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q10" s="0" t="n">
@@ -1785,7 +1785,7 @@
         <v>1.056314</v>
       </c>
       <c r="D11" s="0" t="n">
-        <v>25.700126</v>
+        <v>49.793995</v>
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
@@ -1824,7 +1824,7 @@
       <c r="O11" s="0" t="n"/>
       <c r="P11" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=5 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=5 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q11" s="0" t="n">
@@ -1839,7 +1839,7 @@
         <v>1.006014</v>
       </c>
       <c r="D12" s="0" t="n">
-        <v>72.751122</v>
+        <v>140.955298</v>
       </c>
       <c r="E12" s="0" t="inlineStr">
         <is>
@@ -1878,7 +1878,7 @@
       <c r="O12" s="0" t="n"/>
       <c r="P12" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=5 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=5 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q12" s="0" t="n">
@@ -1893,7 +1893,7 @@
         <v>1.006014</v>
       </c>
       <c r="D13" s="0" t="n">
-        <v>84.34912799999999</v>
+        <v>92.994913</v>
       </c>
       <c r="E13" s="0" t="inlineStr">
         <is>
@@ -1932,7 +1932,7 @@
       <c r="O13" s="0" t="n"/>
       <c r="P13" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=5 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=5 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q13" s="0" t="n">
@@ -1947,7 +1947,7 @@
         <v>1.108275</v>
       </c>
       <c r="D14" s="0" t="n">
-        <v>36.324081</v>
+        <v>70.37790699999999</v>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
@@ -1986,7 +1986,7 @@
       <c r="O14" s="0" t="n"/>
       <c r="P14" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=6 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=6 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q14" s="0" t="n">
@@ -2001,7 +2001,7 @@
         <v>1.057899</v>
       </c>
       <c r="D15" s="0" t="n">
-        <v>23.610651</v>
+        <v>45.745637</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
@@ -2040,7 +2040,7 @@
       <c r="O15" s="0" t="n"/>
       <c r="P15" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=6 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=6 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q15" s="0" t="n">
@@ -2055,7 +2055,7 @@
         <v>1.007523</v>
       </c>
       <c r="D16" s="0" t="n">
-        <v>66.836309</v>
+        <v>129.495348</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
@@ -2094,7 +2094,7 @@
       <c r="O16" s="0" t="n"/>
       <c r="P16" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=6 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=6 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q16" s="0" t="n">
@@ -2109,7 +2109,7 @@
         <v>1.007523</v>
       </c>
       <c r="D17" s="0" t="n">
-        <v>77.491372</v>
+        <v>85.43423799999999</v>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
       <c r="O17" s="0" t="n"/>
       <c r="P17" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=6 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=6 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q17" s="0" t="n">
@@ -2163,7 +2163,7 @@
         <v>1.109937</v>
       </c>
       <c r="D18" s="0" t="n">
-        <v>38.479591</v>
+        <v>74.554208</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
@@ -2202,7 +2202,7 @@
       <c r="O18" s="0" t="n"/>
       <c r="P18" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=7 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | gold20-20261029: reward +20% | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=7 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | gold20-20261029: reward +20% | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q18" s="0" t="n">
@@ -2217,7 +2217,7 @@
         <v>1.059486</v>
       </c>
       <c r="D19" s="0" t="n">
-        <v>25.011736</v>
+        <v>48.460239</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
@@ -2256,7 +2256,7 @@
       <c r="O19" s="0" t="n"/>
       <c r="P19" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=7 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=7 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q19" s="0" t="n">
@@ -2271,7 +2271,7 @@
         <v>1.009034</v>
       </c>
       <c r="D20" s="0" t="n">
-        <v>70.802449</v>
+        <v>137.179745</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
       <c r="O20" s="0" t="n"/>
       <c r="P20" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=7 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=7 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q20" s="0" t="n">
@@ -2325,7 +2325,7 @@
         <v>1.009034</v>
       </c>
       <c r="D21" s="0" t="n">
-        <v>82.08979600000001</v>
+        <v>90.504</v>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
@@ -2364,7 +2364,7 @@
       <c r="O21" s="0" t="n"/>
       <c r="P21" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=7 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=7 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q21" s="0" t="n">
@@ -2379,7 +2379,7 @@
         <v>1.111602</v>
       </c>
       <c r="D22" s="0" t="n">
-        <v>45.95625</v>
+        <v>89.040234</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
@@ -2418,7 +2418,7 @@
       <c r="O22" s="0" t="n"/>
       <c r="P22" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=8 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=8 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q22" s="0" t="n">
@@ -2433,7 +2433,7 @@
         <v>1.061075</v>
       </c>
       <c r="D23" s="0" t="n">
-        <v>29.871562</v>
+        <v>57.876152</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
       <c r="O23" s="0" t="n"/>
       <c r="P23" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=8 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=8 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q23" s="0" t="n">
@@ -2487,7 +2487,7 @@
         <v>1.010547</v>
       </c>
       <c r="D24" s="0" t="n">
-        <v>84.5595</v>
+        <v>163.834031</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
@@ -2526,7 +2526,7 @@
       <c r="O24" s="0" t="n"/>
       <c r="P24" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=8 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=8 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q24" s="0" t="n">
@@ -2541,7 +2541,7 @@
         <v>1.010547</v>
       </c>
       <c r="D25" s="0" t="n">
-        <v>98.04000000000001</v>
+        <v>108.0891</v>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
@@ -2580,7 +2580,7 @@
       <c r="O25" s="0" t="n"/>
       <c r="P25" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=8 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=8 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q25" s="0" t="n">
@@ -2595,7 +2595,7 @@
         <v>1.11327</v>
       </c>
       <c r="D26" s="0" t="n">
-        <v>54.248703</v>
+        <v>105.106862</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
@@ -2634,7 +2634,7 @@
       <c r="O26" s="0" t="n"/>
       <c r="P26" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=9 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=9 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q26" s="0" t="n">
@@ -2649,7 +2649,7 @@
         <v>1.062666</v>
       </c>
       <c r="D27" s="0" t="n">
-        <v>35.261658</v>
+        <v>68.319462</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
@@ -2688,7 +2688,7 @@
       <c r="O27" s="0" t="n"/>
       <c r="P27" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=9 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=9 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q27" s="0" t="n">
@@ -2703,7 +2703,7 @@
         <v>1.012063</v>
       </c>
       <c r="D28" s="0" t="n">
-        <v>99.817617</v>
+        <v>193.396633</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
@@ -2742,7 +2742,7 @@
       <c r="O28" s="0" t="n"/>
       <c r="P28" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=9 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=9 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55)</t>
         </is>
       </c>
       <c r="Q28" s="0" t="n">
@@ -2757,7 +2757,7 @@
         <v>1.012063</v>
       </c>
       <c r="D29" s="0" t="n">
-        <v>115.730568</v>
+        <v>127.592951</v>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
@@ -2796,7 +2796,7 @@
       <c r="O29" s="0" t="n"/>
       <c r="P29" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=9 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=9 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q29" s="0" t="n">
@@ -2811,7 +2811,7 @@
         <v>1.114939</v>
       </c>
       <c r="D30" s="0" t="n">
-        <v>93.32619099999999</v>
+        <v>153.696571</v>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
@@ -2850,7 +2850,7 @@
       <c r="O30" s="0" t="n"/>
       <c r="P30" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=10 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=10 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W10 ground x0.85</t>
         </is>
       </c>
       <c r="Q30" s="0" t="n">
@@ -2865,7 +2865,7 @@
         <v>1.06426</v>
       </c>
       <c r="D31" s="0" t="n">
-        <v>60.662025</v>
+        <v>99.902772</v>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
@@ -2904,7 +2904,7 @@
       <c r="O31" s="0" t="n"/>
       <c r="P31" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=10 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=10 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W10 ground x0.85</t>
         </is>
       </c>
       <c r="Q31" s="0" t="n">
@@ -2919,7 +2919,7 @@
         <v>1.013581</v>
       </c>
       <c r="D32" s="0" t="n">
-        <v>171.720193</v>
+        <v>282.801693</v>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
@@ -2958,7 +2958,7 @@
       <c r="O32" s="0" t="n"/>
       <c r="P32" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=10 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=10 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W10 ground x0.85</t>
         </is>
       </c>
       <c r="Q32" s="0" t="n">
@@ -2973,7 +2973,7 @@
         <v>1.013581</v>
       </c>
       <c r="D33" s="0" t="n">
-        <v>199.095876</v>
+        <v>219.503204</v>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
@@ -3012,7 +3012,7 @@
       <c r="O33" s="0" t="n"/>
       <c r="P33" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=10 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=10 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q33" s="0" t="n">
@@ -3027,7 +3027,7 @@
         <v>1.116612</v>
       </c>
       <c r="D34" s="0" t="n">
-        <v>71.084868</v>
+        <v>117.067892</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
@@ -3066,7 +3066,7 @@
       <c r="O34" s="0" t="n"/>
       <c r="P34" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=11 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=11 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q34" s="0" t="n">
@@ -3081,7 +3081,7 @@
         <v>1.065857</v>
       </c>
       <c r="D35" s="0" t="n">
-        <v>46.205166</v>
+        <v>76.094132</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
@@ -3120,7 +3120,7 @@
       <c r="O35" s="0" t="n"/>
       <c r="P35" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=11 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=11 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q35" s="0" t="n">
@@ -3135,7 +3135,7 @@
         <v>1.015102</v>
       </c>
       <c r="D36" s="0" t="n">
-        <v>130.796157</v>
+        <v>215.404921</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
@@ -3174,7 +3174,7 @@
       <c r="O36" s="0" t="n"/>
       <c r="P36" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=11 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=11 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q36" s="0" t="n">
@@ -3189,7 +3189,7 @@
         <v>0.8120810000000001</v>
       </c>
       <c r="D37" s="0" t="n">
-        <v>241.688551</v>
+        <v>398.030833</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
@@ -3228,7 +3228,7 @@
       <c r="O37" s="0" t="n"/>
       <c r="P37" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=11 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=11 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q37" s="0" t="n">
@@ -3243,7 +3243,7 @@
         <v>1.015102</v>
       </c>
       <c r="D38" s="0" t="n">
-        <v>151.64772</v>
+        <v>167.191611</v>
       </c>
       <c r="E38" s="0" t="inlineStr">
         <is>
@@ -3282,7 +3282,7 @@
       <c r="O38" s="0" t="n"/>
       <c r="P38" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=11 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=11 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q38" s="0" t="n">
@@ -3297,7 +3297,7 @@
         <v>1.118287</v>
       </c>
       <c r="D39" s="0" t="n">
-        <v>68.259739</v>
+        <v>112.415258</v>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
@@ -3336,7 +3336,7 @@
       <c r="O39" s="0" t="n"/>
       <c r="P39" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=12 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=12 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q39" s="0" t="n">
@@ -3351,7 +3351,7 @@
         <v>1.067456</v>
       </c>
       <c r="D40" s="0" t="n">
-        <v>44.368831</v>
+        <v>73.069918</v>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
@@ -3390,7 +3390,7 @@
       <c r="O40" s="0" t="n"/>
       <c r="P40" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=12 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=12 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q40" s="0" t="n">
@@ -3405,7 +3405,7 @@
         <v>1.016624</v>
       </c>
       <c r="D41" s="0" t="n">
-        <v>125.597924</v>
+        <v>206.844081</v>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
@@ -3444,7 +3444,7 @@
       <c r="O41" s="0" t="n"/>
       <c r="P41" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=12 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=12 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q41" s="0" t="n">
@@ -3459,7 +3459,7 @@
         <v>0.813299</v>
       </c>
       <c r="D42" s="0" t="n">
-        <v>232.083117</v>
+        <v>382.211883</v>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
       <c r="O42" s="0" t="n"/>
       <c r="P42" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=12 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=12 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q42" s="0" t="n">
@@ -3513,7 +3513,7 @@
         <v>1.016624</v>
       </c>
       <c r="D43" s="0" t="n">
-        <v>145.62078</v>
+        <v>160.54691</v>
       </c>
       <c r="E43" s="0" t="inlineStr">
         <is>
@@ -3552,7 +3552,7 @@
       <c r="O43" s="0" t="n"/>
       <c r="P43" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=12 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=12 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q43" s="0" t="n">
@@ -3567,7 +3567,7 @@
         <v>1.119964</v>
       </c>
       <c r="D44" s="0" t="n">
-        <v>78.298429</v>
+        <v>128.947725</v>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
@@ -3606,7 +3606,7 @@
       <c r="O44" s="0" t="n"/>
       <c r="P44" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=13 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=13 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q44" s="0" t="n">
@@ -3621,7 +3621,7 @@
         <v>1.069057</v>
       </c>
       <c r="D45" s="0" t="n">
-        <v>50.893979</v>
+        <v>83.816022</v>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
@@ -3660,7 +3660,7 @@
       <c r="O45" s="0" t="n"/>
       <c r="P45" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=13 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=13 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q45" s="0" t="n">
@@ -3675,7 +3675,7 @@
         <v>1.018149</v>
       </c>
       <c r="D46" s="0" t="n">
-        <v>144.069111</v>
+        <v>237.263818</v>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
@@ -3714,7 +3714,7 @@
       <c r="O46" s="0" t="n"/>
       <c r="P46" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=13 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=13 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q46" s="0" t="n">
@@ -3729,7 +3729,7 @@
         <v>0.814519</v>
       </c>
       <c r="D47" s="0" t="n">
-        <v>266.21466</v>
+        <v>438.422268</v>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
@@ -3768,7 +3768,7 @@
       <c r="O47" s="0" t="n"/>
       <c r="P47" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=13 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=13 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q47" s="0" t="n">
@@ -3783,7 +3783,7 @@
         <v>1.018149</v>
       </c>
       <c r="D48" s="0" t="n">
-        <v>167.036648</v>
+        <v>184.157904</v>
       </c>
       <c r="E48" s="0" t="inlineStr">
         <is>
@@ -3822,7 +3822,7 @@
       <c r="O48" s="0" t="n"/>
       <c r="P48" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=13 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=13 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q48" s="0" t="n">
@@ -3837,7 +3837,7 @@
         <v>1.121644</v>
       </c>
       <c r="D49" s="0" t="n">
-        <v>90.25483</v>
+        <v>148.638422</v>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
@@ -3876,7 +3876,7 @@
       <c r="O49" s="0" t="n"/>
       <c r="P49" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=14 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=14 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q49" s="0" t="n">
@@ -3891,7 +3891,7 @@
         <v>1.07066</v>
       </c>
       <c r="D50" s="0" t="n">
-        <v>58.665641</v>
+        <v>96.614977</v>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
@@ -3930,7 +3930,7 @@
       <c r="O50" s="0" t="n"/>
       <c r="P50" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=14 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=14 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q50" s="0" t="n">
@@ -3945,7 +3945,7 @@
         <v>1.019676</v>
       </c>
       <c r="D51" s="0" t="n">
-        <v>166.068887</v>
+        <v>273.494699</v>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
@@ -3984,7 +3984,7 @@
       <c r="O51" s="0" t="n"/>
       <c r="P51" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=14 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=14 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q51" s="0" t="n">
@@ -3999,7 +3999,7 @@
         <v>0.815741</v>
       </c>
       <c r="D52" s="0" t="n">
-        <v>306.866422</v>
+        <v>505.370639</v>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
@@ -4038,7 +4038,7 @@
       <c r="O52" s="0" t="n"/>
       <c r="P52" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=14 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=14 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85)</t>
         </is>
       </c>
       <c r="Q52" s="0" t="n">
@@ -4053,7 +4053,7 @@
         <v>1.019676</v>
       </c>
       <c r="D53" s="0" t="n">
-        <v>192.543636</v>
+        <v>212.279359</v>
       </c>
       <c r="E53" s="0" t="inlineStr">
         <is>
@@ -4092,7 +4092,7 @@
       <c r="O53" s="0" t="n"/>
       <c r="P53" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=14 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=14 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q53" s="0" t="n">
@@ -4107,7 +4107,7 @@
         <v>1.123327</v>
       </c>
       <c r="D54" s="0" t="n">
-        <v>147.857144</v>
+        <v>208.19441</v>
       </c>
       <c r="E54" s="0" t="inlineStr">
         <is>
@@ -4146,7 +4146,7 @@
       <c r="O54" s="0" t="n"/>
       <c r="P54" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=15 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=15 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q54" s="0" t="n">
@@ -4161,7 +4161,7 @@
         <v>1.072266</v>
       </c>
       <c r="D55" s="0" t="n">
-        <v>96.10714299999999</v>
+        <v>135.326367</v>
       </c>
       <c r="E55" s="0" t="inlineStr">
         <is>
@@ -4200,7 +4200,7 @@
       <c r="O55" s="0" t="n"/>
       <c r="P55" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=15 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=15 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q55" s="0" t="n">
@@ -4215,7 +4215,7 @@
         <v>1.021206</v>
       </c>
       <c r="D56" s="0" t="n">
-        <v>272.057143</v>
+        <v>383.077712</v>
       </c>
       <c r="E56" s="0" t="inlineStr">
         <is>
@@ -4254,7 +4254,7 @@
       <c r="O56" s="0" t="n"/>
       <c r="P56" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=15 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=15 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q56" s="0" t="n">
@@ -4269,7 +4269,7 @@
         <v>0.8169650000000001</v>
       </c>
       <c r="D57" s="0" t="n">
-        <v>502.714284</v>
+        <v>707.860986</v>
       </c>
       <c r="E57" s="0" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       <c r="O57" s="0" t="n"/>
       <c r="P57" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=15 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=15 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q57" s="0" t="n">
@@ -4323,7 +4323,7 @@
         <v>1.021206</v>
       </c>
       <c r="D58" s="0" t="n">
-        <v>315.428572</v>
+        <v>347.760001</v>
       </c>
       <c r="E58" s="0" t="inlineStr">
         <is>
@@ -4362,7 +4362,7 @@
       <c r="O58" s="0" t="n"/>
       <c r="P58" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=15 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=15 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q58" s="0" t="n">
@@ -4377,7 +4377,7 @@
         <v>1.125012</v>
       </c>
       <c r="D59" s="0" t="n">
-        <v>144.948933</v>
+        <v>204.099421</v>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
@@ -4416,7 +4416,7 @@
       <c r="O59" s="0" t="n"/>
       <c r="P59" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=16 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=16 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q59" s="0" t="n">
@@ -4431,7 +4431,7 @@
         <v>1.073875</v>
       </c>
       <c r="D60" s="0" t="n">
-        <v>94.21680600000001</v>
+        <v>132.664624</v>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
@@ -4470,7 +4470,7 @@
       <c r="O60" s="0" t="n"/>
       <c r="P60" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=16 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=16 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q60" s="0" t="n">
@@ -4485,7 +4485,7 @@
         <v>1.022738</v>
       </c>
       <c r="D61" s="0" t="n">
-        <v>266.706037</v>
+        <v>375.542936</v>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
@@ -4524,7 +4524,7 @@
       <c r="O61" s="0" t="n"/>
       <c r="P61" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=16 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=16 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q61" s="0" t="n">
@@ -4539,7 +4539,7 @@
         <v>0.81819</v>
       </c>
       <c r="D62" s="0" t="n">
-        <v>492.826374</v>
+        <v>693.938036</v>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
@@ -4578,7 +4578,7 @@
       <c r="O62" s="0" t="n"/>
       <c r="P62" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=16 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=16 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q62" s="0" t="n">
@@ -4593,7 +4593,7 @@
         <v>1.022738</v>
       </c>
       <c r="D63" s="0" t="n">
-        <v>309.224392</v>
+        <v>340.919893</v>
       </c>
       <c r="E63" s="0" t="inlineStr">
         <is>
@@ -4632,7 +4632,7 @@
       <c r="O63" s="0" t="n"/>
       <c r="P63" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=16 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=16 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q63" s="0" t="n">
@@ -4647,7 +4647,7 @@
         <v>1.126699</v>
       </c>
       <c r="D64" s="0" t="n">
-        <v>139.53063</v>
+        <v>196.470027</v>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
@@ -4686,7 +4686,7 @@
       <c r="O64" s="0" t="n"/>
       <c r="P64" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=17 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=17 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q64" s="0" t="n">
@@ -4701,7 +4701,7 @@
         <v>1.075485</v>
       </c>
       <c r="D65" s="0" t="n">
-        <v>90.694909</v>
+        <v>127.705517</v>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
@@ -4740,7 +4740,7 @@
       <c r="O65" s="0" t="n"/>
       <c r="P65" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=17 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=17 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q65" s="0" t="n">
@@ -4755,7 +4755,7 @@
         <v>1.024272</v>
       </c>
       <c r="D66" s="0" t="n">
-        <v>256.736358</v>
+        <v>361.50485</v>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       <c r="O66" s="0" t="n"/>
       <c r="P66" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=17 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=17 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q66" s="0" t="n">
@@ -4809,7 +4809,7 @@
         <v>0.819418</v>
       </c>
       <c r="D67" s="0" t="n">
-        <v>474.404142</v>
+        <v>667.998094</v>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
       <c r="O67" s="0" t="n"/>
       <c r="P67" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=17 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=17 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q67" s="0" t="n">
@@ -4863,7 +4863,7 @@
         <v>1.024272</v>
       </c>
       <c r="D68" s="0" t="n">
-        <v>297.665344</v>
+        <v>328.176042</v>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
@@ -4902,7 +4902,7 @@
       <c r="O68" s="0" t="n"/>
       <c r="P68" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=17 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=17 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q68" s="0" t="n">
@@ -4917,7 +4917,7 @@
         <v>1.128389</v>
       </c>
       <c r="D69" s="0" t="n">
-        <v>142.036187</v>
+        <v>199.998048</v>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
@@ -4956,7 +4956,7 @@
       <c r="O69" s="0" t="n"/>
       <c r="P69" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=18 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=18 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q69" s="0" t="n">
@@ -4971,7 +4971,7 @@
         <v>1.077099</v>
       </c>
       <c r="D70" s="0" t="n">
-        <v>92.323521</v>
+        <v>129.998731</v>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
@@ -5010,7 +5010,7 @@
       <c r="O70" s="0" t="n"/>
       <c r="P70" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=18 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=18 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q70" s="0" t="n">
@@ -5025,7 +5025,7 @@
         <v>1.025808</v>
       </c>
       <c r="D71" s="0" t="n">
-        <v>261.346583</v>
+        <v>367.996407</v>
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
@@ -5064,7 +5064,7 @@
       <c r="O71" s="0" t="n"/>
       <c r="P71" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=18 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=18 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q71" s="0" t="n">
@@ -5079,7 +5079,7 @@
         <v>0.820647</v>
       </c>
       <c r="D72" s="0" t="n">
-        <v>482.923035</v>
+        <v>679.993363</v>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
@@ -5118,7 +5118,7 @@
       <c r="O72" s="0" t="n"/>
       <c r="P72" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=18 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=18 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q72" s="0" t="n">
@@ -5133,7 +5133,7 @@
         <v>1.025808</v>
       </c>
       <c r="D73" s="0" t="n">
-        <v>303.010532</v>
+        <v>334.069112</v>
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
@@ -5172,7 +5172,7 @@
       <c r="O73" s="0" t="n"/>
       <c r="P73" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=18 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=18 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q73" s="0" t="n">
@@ -5187,7 +5187,7 @@
         <v>1.130082</v>
       </c>
       <c r="D74" s="0" t="n">
-        <v>158.949909</v>
+        <v>223.81389</v>
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
@@ -5226,7 +5226,7 @@
       <c r="O74" s="0" t="n"/>
       <c r="P74" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=19 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=19 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q74" s="0" t="n">
@@ -5241,7 +5241,7 @@
         <v>1.078714</v>
       </c>
       <c r="D75" s="0" t="n">
-        <v>103.317442</v>
+        <v>145.479031</v>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
@@ -5280,7 +5280,7 @@
       <c r="O75" s="0" t="n"/>
       <c r="P75" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=19 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=19 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q75" s="0" t="n">
@@ -5295,7 +5295,7 @@
         <v>1.027347</v>
       </c>
       <c r="D76" s="0" t="n">
-        <v>292.467832</v>
+        <v>411.817556</v>
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
@@ -5334,7 +5334,7 @@
       <c r="O76" s="0" t="n"/>
       <c r="P76" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=19 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=19 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q76" s="0" t="n">
@@ -5349,7 +5349,7 @@
         <v>0.821878</v>
       </c>
       <c r="D77" s="0" t="n">
-        <v>540.4296900000001</v>
+        <v>760.967224</v>
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
@@ -5388,7 +5388,7 @@
       <c r="O77" s="0" t="n"/>
       <c r="P77" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=19 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=19 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q77" s="0" t="n">
@@ -5403,7 +5403,7 @@
         <v>1.027347</v>
       </c>
       <c r="D78" s="0" t="n">
-        <v>339.09314</v>
+        <v>373.850187</v>
       </c>
       <c r="E78" s="0" t="inlineStr">
         <is>
@@ -5442,7 +5442,7 @@
       <c r="O78" s="0" t="n"/>
       <c r="P78" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=19 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=19 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q78" s="0" t="n">
@@ -5457,7 +5457,7 @@
         <v>1.131777</v>
       </c>
       <c r="D79" s="0" t="n">
-        <v>196.383942</v>
+        <v>276.523933</v>
       </c>
       <c r="E79" s="0" t="inlineStr">
         <is>
@@ -5496,7 +5496,7 @@
       <c r="O79" s="0" t="n"/>
       <c r="P79" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | w20soften-20261029: hp x0.7736 | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | w20soften-20261029: hp x0.7736 | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q79" s="0" t="n">
@@ -5511,7 +5511,7 @@
         <v>1.080332</v>
       </c>
       <c r="D80" s="0" t="n">
-        <v>127.649561</v>
+        <v>179.740554</v>
       </c>
       <c r="E80" s="0" t="inlineStr">
         <is>
@@ -5550,7 +5550,7 @@
       <c r="O80" s="0" t="n"/>
       <c r="P80" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | w20soften-20261029: hp x0.7736 | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | w20soften-20261029: hp x0.7736 | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q80" s="0" t="n">
@@ -5565,7 +5565,7 @@
         <v>1.028888</v>
       </c>
       <c r="D81" s="0" t="n">
-        <v>361.346452</v>
+        <v>508.804034</v>
       </c>
       <c r="E81" s="0" t="inlineStr">
         <is>
@@ -5604,7 +5604,7 @@
       <c r="O81" s="0" t="n"/>
       <c r="P81" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | w20soften-20261029: hp x0.7736 | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | w20soften-20261029: hp x0.7736 | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q81" s="0" t="n">
@@ -5619,7 +5619,7 @@
         <v>0.82311</v>
       </c>
       <c r="D82" s="0" t="n">
-        <v>667.7053990000001</v>
+        <v>940.181366</v>
       </c>
       <c r="E82" s="0" t="inlineStr">
         <is>
@@ -5658,7 +5658,7 @@
       <c r="O82" s="0" t="n"/>
       <c r="P82" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | w20soften-20261029: hp x0.7736 | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | w20soften-20261029: hp x0.7736 | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q82" s="0" t="n">
@@ -5673,7 +5673,7 @@
         <v>1.028888</v>
       </c>
       <c r="D83" s="0" t="n">
-        <v>418.952407</v>
+        <v>461.895028</v>
       </c>
       <c r="E83" s="0" t="inlineStr">
         <is>
@@ -5712,7 +5712,7 @@
       <c r="O83" s="0" t="n"/>
       <c r="P83" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | w20soften-20261029: hp x0.7736</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | w20soften-20261029: hp x0.7736 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q83" s="0" t="n">
@@ -5727,7 +5727,7 @@
         <v>1.133475</v>
       </c>
       <c r="D84" s="0" t="n">
-        <v>250.453564</v>
+        <v>352.658185</v>
       </c>
       <c r="E84" s="0" t="inlineStr">
         <is>
@@ -5766,7 +5766,7 @@
       <c r="O84" s="0" t="n"/>
       <c r="P84" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q84" s="0" t="n">
@@ -5781,7 +5781,7 @@
         <v>1.081953</v>
       </c>
       <c r="D85" s="0" t="n">
-        <v>162.794817</v>
+        <v>229.227821</v>
       </c>
       <c r="E85" s="0" t="inlineStr">
         <is>
@@ -5820,7 +5820,7 @@
       <c r="O85" s="0" t="n"/>
       <c r="P85" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q85" s="0" t="n">
@@ -5835,7 +5835,7 @@
         <v>1.030431</v>
       </c>
       <c r="D86" s="0" t="n">
-        <v>460.834559</v>
+        <v>648.891062</v>
       </c>
       <c r="E86" s="0" t="inlineStr">
         <is>
@@ -5874,7 +5874,7 @@
       <c r="O86" s="0" t="n"/>
       <c r="P86" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q86" s="0" t="n">
@@ -5889,7 +5889,7 @@
         <v>0.824345</v>
       </c>
       <c r="D87" s="0" t="n">
-        <v>851.542118</v>
+        <v>1199.037828</v>
       </c>
       <c r="E87" s="0" t="inlineStr">
         <is>
@@ -5928,7 +5928,7 @@
       <c r="O87" s="0" t="n"/>
       <c r="P87" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q87" s="0" t="n">
@@ -5943,7 +5943,7 @@
         <v>1.030431</v>
       </c>
       <c r="D88" s="0" t="n">
-        <v>507.585889</v>
+        <v>559.613442</v>
       </c>
       <c r="E88" s="0" t="inlineStr">
         <is>
@@ -5982,7 +5982,7 @@
       <c r="O88" s="0" t="n"/>
       <c r="P88" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q88" s="0" t="n">
@@ -5997,7 +5997,7 @@
         <v>1.135175</v>
       </c>
       <c r="D89" s="0" t="n">
-        <v>244.375718</v>
+        <v>344.100103</v>
       </c>
       <c r="E89" s="0" t="inlineStr">
         <is>
@@ -6036,7 +6036,7 @@
       <c r="O89" s="0" t="n"/>
       <c r="P89" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q89" s="0" t="n">
@@ -6051,7 +6051,7 @@
         <v>1.083576</v>
       </c>
       <c r="D90" s="0" t="n">
-        <v>158.844216</v>
+        <v>223.665066</v>
       </c>
       <c r="E90" s="0" t="inlineStr">
         <is>
@@ -6090,7 +6090,7 @@
       <c r="O90" s="0" t="n"/>
       <c r="P90" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q90" s="0" t="n">
@@ -6105,7 +6105,7 @@
         <v>1.031977</v>
       </c>
       <c r="D91" s="0" t="n">
-        <v>449.651319</v>
+        <v>633.144186</v>
       </c>
       <c r="E91" s="0" t="inlineStr">
         <is>
@@ -6144,7 +6144,7 @@
       <c r="O91" s="0" t="n"/>
       <c r="P91" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q91" s="0" t="n">
@@ -6159,7 +6159,7 @@
         <v>0.825582</v>
       </c>
       <c r="D92" s="0" t="n">
-        <v>830.877439</v>
+        <v>1169.940346</v>
       </c>
       <c r="E92" s="0" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
       <c r="O92" s="0" t="n"/>
       <c r="P92" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q92" s="0" t="n">
@@ -6213,7 +6213,7 @@
         <v>1.031977</v>
       </c>
       <c r="D93" s="0" t="n">
-        <v>495.268121</v>
+        <v>546.033103</v>
       </c>
       <c r="E93" s="0" t="inlineStr">
         <is>
@@ -6252,7 +6252,7 @@
       <c r="O93" s="0" t="n"/>
       <c r="P93" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q93" s="0" t="n">
@@ -6267,7 +6267,7 @@
         <v>1.136877</v>
       </c>
       <c r="D94" s="0" t="n">
-        <v>239.569916</v>
+        <v>337.333158</v>
       </c>
       <c r="E94" s="0" t="inlineStr">
         <is>
@@ -6306,7 +6306,7 @@
       <c r="O94" s="0" t="n"/>
       <c r="P94" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=23 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=23 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q94" s="0" t="n">
@@ -6321,7 +6321,7 @@
         <v>1.085201</v>
       </c>
       <c r="D95" s="0" t="n">
-        <v>155.720445</v>
+        <v>219.266552</v>
       </c>
       <c r="E95" s="0" t="inlineStr">
         <is>
@@ -6360,7 +6360,7 @@
       <c r="O95" s="0" t="n"/>
       <c r="P95" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=23 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=23 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q95" s="0" t="n">
@@ -6375,7 +6375,7 @@
         <v>1.033525</v>
       </c>
       <c r="D96" s="0" t="n">
-        <v>440.808647</v>
+        <v>620.6930139999999</v>
       </c>
       <c r="E96" s="0" t="inlineStr">
         <is>
@@ -6414,7 +6414,7 @@
       <c r="O96" s="0" t="n"/>
       <c r="P96" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=23 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=23 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q96" s="0" t="n">
@@ -6429,7 +6429,7 @@
         <v>0.82682</v>
       </c>
       <c r="D97" s="0" t="n">
-        <v>814.5377140000001</v>
+        <v>1146.932738</v>
       </c>
       <c r="E97" s="0" t="inlineStr">
         <is>
@@ -6468,7 +6468,7 @@
       <c r="O97" s="0" t="n"/>
       <c r="P97" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=23 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=23 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q97" s="0" t="n">
@@ -6483,7 +6483,7 @@
         <v>1.033525</v>
       </c>
       <c r="D98" s="0" t="n">
-        <v>485.528364</v>
+        <v>535.295021</v>
       </c>
       <c r="E98" s="0" t="inlineStr">
         <is>
@@ -6522,7 +6522,7 @@
       <c r="O98" s="0" t="n"/>
       <c r="P98" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=23 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=23 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q98" s="0" t="n">
@@ -6537,7 +6537,7 @@
         <v>1.138583</v>
       </c>
       <c r="D99" s="0" t="n">
-        <v>248.921001</v>
+        <v>350.500216</v>
       </c>
       <c r="E99" s="0" t="inlineStr">
         <is>
@@ -6576,7 +6576,7 @@
       <c r="O99" s="0" t="n"/>
       <c r="P99" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=24 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | gold20-20261029: reward +20% | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1909 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=24 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | gold20-20261029: reward +20% | flatdrop-20261029: 0.20/只(角色=normal) | econneutral-20261030: 0.1909 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q99" s="0" t="n">
@@ -6591,7 +6591,7 @@
         <v>1.086829</v>
       </c>
       <c r="D100" s="0" t="n">
-        <v>161.798652</v>
+        <v>227.825143</v>
       </c>
       <c r="E100" s="0" t="inlineStr">
         <is>
@@ -6630,7 +6630,7 @@
       <c r="O100" s="0" t="n"/>
       <c r="P100" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=24 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=24 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q100" s="0" t="n">
@@ -6645,7 +6645,7 @@
         <v>1.035075</v>
       </c>
       <c r="D101" s="0" t="n">
-        <v>458.014644</v>
+        <v>644.920401</v>
       </c>
       <c r="E101" s="0" t="inlineStr">
         <is>
@@ -6684,7 +6684,7 @@
       <c r="O101" s="0" t="n"/>
       <c r="P101" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=24 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=24 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q101" s="0" t="n">
@@ -6699,7 +6699,7 @@
         <v>0.82806</v>
       </c>
       <c r="D102" s="0" t="n">
-        <v>846.331407</v>
+        <v>1191.70074</v>
       </c>
       <c r="E102" s="0" t="inlineStr">
         <is>
@@ -6738,7 +6738,7 @@
       <c r="O102" s="0" t="n"/>
       <c r="P102" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=24 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=24 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q102" s="0" t="n">
@@ -6753,7 +6753,7 @@
         <v>1.035075</v>
       </c>
       <c r="D103" s="0" t="n">
-        <v>504.479898</v>
+        <v>556.189088</v>
       </c>
       <c r="E103" s="0" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
       <c r="O103" s="0" t="n"/>
       <c r="P103" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=24 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=24 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q103" s="0" t="n">
@@ -6807,7 +6807,7 @@
         <v>1.140291</v>
       </c>
       <c r="D104" s="0" t="n">
-        <v>342.907479</v>
+        <v>482.840521</v>
       </c>
       <c r="E104" s="0" t="inlineStr">
         <is>
@@ -6846,7 +6846,7 @@
       <c r="O104" s="0" t="n"/>
       <c r="P104" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.1903 (was 0.20)</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q104" s="0" t="n">
@@ -6861,7 +6861,7 @@
         <v>1.088459</v>
       </c>
       <c r="D105" s="0" t="n">
-        <v>222.889862</v>
+        <v>313.846339</v>
       </c>
       <c r="E105" s="0" t="inlineStr">
         <is>
@@ -6900,7 +6900,7 @@
       <c r="O105" s="0" t="n"/>
       <c r="P105" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.1522 (was 0.16)</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q105" s="0" t="n">
@@ -6915,7 +6915,7 @@
         <v>1.036628</v>
       </c>
       <c r="D106" s="0" t="n">
-        <v>630.949761</v>
+        <v>888.426557</v>
       </c>
       <c r="E106" s="0" t="inlineStr">
         <is>
@@ -6954,7 +6954,7 @@
       <c r="O106" s="0" t="n"/>
       <c r="P106" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.3045 (was 0.32)</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q106" s="0" t="n">
@@ -6969,7 +6969,7 @@
         <v>0.829302</v>
       </c>
       <c r="D107" s="0" t="n">
-        <v>1165.885428</v>
+        <v>1641.657768</v>
       </c>
       <c r="E107" s="0" t="inlineStr">
         <is>
@@ -7008,7 +7008,7 @@
       <c r="O107" s="0" t="n"/>
       <c r="P107" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.4948 (was 0.52)</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q107" s="0" t="n">
@@ -7023,7 +7023,7 @@
         <v>0.777471</v>
       </c>
       <c r="D108" s="0" t="n">
-        <v>1872.274838</v>
+        <v>2636.309244</v>
       </c>
       <c r="E108" s="0" t="inlineStr">
         <is>
@@ -7062,7 +7062,7 @@
       <c r="O108" s="0" t="n"/>
       <c r="P108" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=123; role=elite; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 1.40/只(角色=elite) | w25soften-20261030: hp x0.80 | econneutral-20261030: 1.3322 (was 1.40)</t>
+          <t>Balance variant; canonical=123; role=elite; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 1.40/只(角色=elite) | w25soften-20261030: hp x0.80 | econneutral-20261030: 1.3322 (was 1.40) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
         </is>
       </c>
       <c r="Q108" s="0" t="n">
@@ -7077,7 +7077,7 @@
         <v>1.036628</v>
       </c>
       <c r="D109" s="0" t="n">
-        <v>694.959158</v>
+        <v>766.192472</v>
       </c>
       <c r="E109" s="0" t="inlineStr">
         <is>
@@ -7116,7 +7116,7 @@
       <c r="O109" s="0" t="n"/>
       <c r="P109" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95 | w25soften-20261030: hp x0.80</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95 | w25soften-20261030: hp x0.80 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
         </is>
       </c>
       <c r="Q109" s="0" t="n">

</xml_diff>

<commit_message>
feat(balance): L01 W20/W21 空中怪四轮 -5%，重封 30 关评级哈希
- EnemyData.xlsx：W20 Bat(5000195) hp 461.895028→438.800277；
  W21 Bat(5000205) 559.613442→455.808646（四轮 ×0.95，累计 -18.55%），desc 逐轮追加
- EnemyList.xlsx：W20/W21 desc 追加 airhp*-20261031 与对应 EHP
  （W20 241829.747662→240259.304594、W21 314172.079845→307217.158513）
- Luban 导出：tbenemydata.json 4 行、tbenemylist.json 2 行；
  Assets/Gen/*.cs 仅行尾差异，无内容变化（导出会删 FTProject.Gen.asmdef，已按惯例还原）
- 30 张 Levels/Lxx/LevelRating.xlsx 重封 runtimeContentHash：全局同值
  cc53b074…→622ae4d4…，算法取 Configs.CalculateRuntimeContentHash（9 张 json + 30 行评级字段）
- 校验：Unity execute_code 复算 stored==recomputed，W20BatHp=438.8003、W21BatHp=455.8087；
  read_console "error CS" 0 条
- 附 .workbuddy/analysis：L01 25 波 EHP/单波压力明细与两张走势图（本轮调参依据）
</commit_message>
<xml_diff>
--- a/Luban/Config/Datas/Levels/L01/EnemyData.xlsx
+++ b/Luban/Config/Datas/Levels/L01/EnemyData.xlsx
@@ -5673,7 +5673,7 @@
         <v>1.028888</v>
       </c>
       <c r="D83" s="0" t="n">
-        <v>461.895028</v>
+        <v>438.800277</v>
       </c>
       <c r="E83" s="0" t="inlineStr">
         <is>
@@ -5712,7 +5712,7 @@
       <c r="O83" s="0" t="n"/>
       <c r="P83" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | w20soften-20261029: hp x0.7736 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=20 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | w20soften-20261029: hp x0.7736 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05) | airhp-20261031: W20 air x0.95</t>
         </is>
       </c>
       <c r="Q83" s="0" t="n">
@@ -5943,7 +5943,7 @@
         <v>1.030431</v>
       </c>
       <c r="D88" s="0" t="n">
-        <v>559.613442</v>
+        <v>455.808646</v>
       </c>
       <c r="E88" s="0" t="inlineStr">
         <is>
@@ -5982,7 +5982,7 @@
       <c r="O88" s="0" t="n"/>
       <c r="P88" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=21 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05) | airhp-20261031: W21 air x0.95 | airhp2-20261031: W21 air x0.95 again | airhp3-20261031: W21 air x0.95 (third) | airhp4-20261031: W21 air x0.95 (fourth)</t>
         </is>
       </c>
       <c r="Q88" s="0" t="n">

</xml_diff>

<commit_message>
feat(balance): L01 第25波地面怪血量 -5%
波次定位：RoundData 的 id 不是顺序波次号，「第 25/25 波」= RoundData id 405
= EnemyList id 405（RoundData 表内顺序为 1..20 → 401..405 → 13..20）。

按用户确认的最小范围，只改 isFlying=0 的 5 种，Bat 不动，reward 不调：

  Chicken 5000240  482.840521 -> 458.698495
  Larva   5000241  313.846339 -> 298.154022
  Crawler 5000242  888.426557 -> 844.005229
  Scarab  5000243 1641.657768 -> 1559.574880
  Rat     5000244 2636.309244 -> 2504.493782
  Bat     5000245  766.192472 -> 未改动（isFlying=1）

EHP：地面部分 496649.76 -> 471817.27（-5.000%），整波 560243.734591 ->
535411.246654（-4.432%，Bat 占该波 11% 权重未动）。

另外两处顺带处理（已与用户确认）：
- EnemyList 405 行首 EHP 汇总原为 410396.243063，是 hp3/hp4/hp5 几轮只更新括号
  分项、漏更行首造成的历史遗留值（真实值应为 560243.734591）。本次按当前 hp/armor
  重算并写明来源，避免后续被误读。
- tbenemydata.json 同时带出 W22 蝙蝠 5000215 的 546.033103 -> 491.429793：
  该改动由上一轮会话改表并导出、只是未提交，本次导出对其幂等，不是本次新增。

每行 desc 追加 hp6-20261101 记录。其余关卡、其余波次未改动。
两个 .bak_20261101_hp6 为改表前的回滚点。
</commit_message>
<xml_diff>
--- a/Luban/Config/Datas/Levels/L01/EnemyData.xlsx
+++ b/Luban/Config/Datas/Levels/L01/EnemyData.xlsx
@@ -6213,7 +6213,7 @@
         <v>1.031977</v>
       </c>
       <c r="D93" s="0" t="n">
-        <v>546.033103</v>
+        <v>491.429793</v>
       </c>
       <c r="E93" s="0" t="inlineStr">
         <is>
@@ -6252,7 +6252,7 @@
       <c r="O93" s="0" t="n"/>
       <c r="P93" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05)</t>
+          <t>Balance variant; canonical=11; role=air; profile=D04; level=1; wave=22 | wavebuff-20261029: hp x2.0, reward per-wave budget | wavebuff2-20261029: hp x2.0 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.36/只(角色=air) | wavegold-air-20261029: hp x0.95 | hp-20261030: ground x1.25, air x1.05 (x1.05) | hp2-20261030: ground x1.55, air x1.05 (x1.05) | airhp-20261101: W22 air x0.90</t>
         </is>
       </c>
       <c r="Q93" s="0" t="n">
@@ -6807,7 +6807,7 @@
         <v>1.140291</v>
       </c>
       <c r="D104" s="0" t="n">
-        <v>482.840521</v>
+        <v>458.698495</v>
       </c>
       <c r="E104" s="0" t="inlineStr">
         <is>
@@ -6846,7 +6846,7 @@
       <c r="O104" s="0" t="n"/>
       <c r="P104" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
+          <t>Balance variant; canonical=18; role=normal; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.20/只(角色=normal) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.1903 (was 0.20) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95 | hp6-20261101: W25 ground x0.95</t>
         </is>
       </c>
       <c r="Q104" s="0" t="n">
@@ -6861,7 +6861,7 @@
         <v>1.088459</v>
       </c>
       <c r="D105" s="0" t="n">
-        <v>313.846339</v>
+        <v>298.154022</v>
       </c>
       <c r="E105" s="0" t="inlineStr">
         <is>
@@ -6900,7 +6900,7 @@
       <c r="O105" s="0" t="n"/>
       <c r="P105" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
+          <t>Balance variant; canonical=84; role=swarm; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.16/只(角色=swarm) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.1522 (was 0.16) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95 | hp6-20261101: W25 ground x0.95</t>
         </is>
       </c>
       <c r="Q105" s="0" t="n">
@@ -6915,7 +6915,7 @@
         <v>1.036628</v>
       </c>
       <c r="D106" s="0" t="n">
-        <v>888.426557</v>
+        <v>844.005229</v>
       </c>
       <c r="E106" s="0" t="inlineStr">
         <is>
@@ -6954,7 +6954,7 @@
       <c r="O106" s="0" t="n"/>
       <c r="P106" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
+          <t>Balance variant; canonical=83; role=medium; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.32/只(角色=medium) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.3045 (was 0.32) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95 | hp6-20261101: W25 ground x0.95</t>
         </is>
       </c>
       <c r="Q106" s="0" t="n">
@@ -6969,7 +6969,7 @@
         <v>0.829302</v>
       </c>
       <c r="D107" s="0" t="n">
-        <v>1641.657768</v>
+        <v>1559.57488</v>
       </c>
       <c r="E107" s="0" t="inlineStr">
         <is>
@@ -7008,7 +7008,7 @@
       <c r="O107" s="0" t="n"/>
       <c r="P107" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
+          <t>Balance variant; canonical=88; role=heavy; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 0.52/只(角色=heavy) | w25soften-20261030: hp x0.80 | econneutral-20261030: 0.4948 (was 0.52) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95 | hp6-20261101: W25 ground x0.95</t>
         </is>
       </c>
       <c r="Q107" s="0" t="n">
@@ -7023,7 +7023,7 @@
         <v>0.777471</v>
       </c>
       <c r="D108" s="0" t="n">
-        <v>2636.309244</v>
+        <v>2504.493782</v>
       </c>
       <c r="E108" s="0" t="inlineStr">
         <is>
@@ -7062,7 +7062,7 @@
       <c r="O108" s="0" t="n"/>
       <c r="P108" s="0" t="inlineStr">
         <is>
-          <t>Balance variant; canonical=123; role=elite; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 1.40/只(角色=elite) | w25soften-20261030: hp x0.80 | econneutral-20261030: 1.3322 (was 1.40) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95</t>
+          <t>Balance variant; canonical=123; role=elite; profile=D04; level=1; wave=25 | wavebuff-20261029: hp x1.5, reward per-wave budget | wavebuff2-20261029: hp x1.5 again, counts x2 again, reward halved-budget | flatdrop-20261029: 1.40/只(角色=elite) | w25soften-20261030: hp x0.80 | econneutral-20261030: 1.3322 (was 1.40) | hp-20261030: ground x1.25, air x1.05 (x1.25) | hp2-20261030: ground x1.55, air x1.05 (x1.55) | hp3-20261030: W11-25 ground x0.85 (ground x0.85) | hp4-20261030: W15-25 ground x0.9 | hp5-20261030: W15-25 ground x0.95 | hp6-20261101: W25 ground x0.95</t>
         </is>
       </c>
       <c r="Q108" s="0" t="n">

</xml_diff>

<commit_message>
feat(balance): L01 地面血量 W6-24 +12%、W25 地面 -5%/空中 +3%
W6/7/8/9/11/12/13/14/16/17/18/19/21/22/23/24 共 16 波的地面变体 hp x1.12（60 行，ratio 全为 1.120000），W10/15/20/25 与全部空军不动；W25 末波另按地面 x0.95、空中 Bat x1.03 调整（6 行），W25 EHP 535411→513728（-4.05%）。EnemyList 同步重算对应波次 EHP 并追加 goldhp/w25hp2 标记。全部改动只落在 L01，hp 以外字段 0 变化。
</commit_message>
<xml_diff>
--- a/Luban/Config/Datas/Levels/L01/EnemyData.xlsx
+++ b/Luban/Config/Datas/Levels/L01/EnemyData.xlsx
@@ -1947,7 +1947,7 @@
         <v>1.108275</v>
       </c>
       <c r="D14" s="0" t="n">
-        <v>70.37790699999999</v>
+        <v>78.823256</v>
       </c>
       <c r="E14" s="0" t="inlineStr">
         <is>
@@ -2001,7 +2001,7 @@
         <v>1.057899</v>
       </c>
       <c r="D15" s="0" t="n">
-        <v>45.745637</v>
+        <v>51.235113</v>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
@@ -2055,7 +2055,7 @@
         <v>1.007523</v>
       </c>
       <c r="D16" s="0" t="n">
-        <v>129.495348</v>
+        <v>145.03479</v>
       </c>
       <c r="E16" s="0" t="inlineStr">
         <is>
@@ -2163,7 +2163,7 @@
         <v>1.109937</v>
       </c>
       <c r="D18" s="0" t="n">
-        <v>74.554208</v>
+        <v>83.500713</v>
       </c>
       <c r="E18" s="0" t="inlineStr">
         <is>
@@ -2217,7 +2217,7 @@
         <v>1.059486</v>
       </c>
       <c r="D19" s="0" t="n">
-        <v>48.460239</v>
+        <v>54.275468</v>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         <v>1.009034</v>
       </c>
       <c r="D20" s="0" t="n">
-        <v>137.179745</v>
+        <v>153.641314</v>
       </c>
       <c r="E20" s="0" t="inlineStr">
         <is>
@@ -2379,7 +2379,7 @@
         <v>1.111602</v>
       </c>
       <c r="D22" s="0" t="n">
-        <v>89.040234</v>
+        <v>99.72506199999999</v>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
         <v>1.061075</v>
       </c>
       <c r="D23" s="0" t="n">
-        <v>57.876152</v>
+        <v>64.82129</v>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
@@ -2487,7 +2487,7 @@
         <v>1.010547</v>
       </c>
       <c r="D24" s="0" t="n">
-        <v>163.834031</v>
+        <v>183.494115</v>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
@@ -2595,7 +2595,7 @@
         <v>1.11327</v>
       </c>
       <c r="D26" s="0" t="n">
-        <v>105.106862</v>
+        <v>117.719685</v>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
@@ -2649,7 +2649,7 @@
         <v>1.062666</v>
       </c>
       <c r="D27" s="0" t="n">
-        <v>68.319462</v>
+        <v>76.517797</v>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
@@ -2703,7 +2703,7 @@
         <v>1.012063</v>
       </c>
       <c r="D28" s="0" t="n">
-        <v>193.396633</v>
+        <v>216.604229</v>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
@@ -3027,7 +3027,7 @@
         <v>1.116612</v>
       </c>
       <c r="D34" s="0" t="n">
-        <v>117.067892</v>
+        <v>131.116039</v>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
@@ -3081,7 +3081,7 @@
         <v>1.065857</v>
       </c>
       <c r="D35" s="0" t="n">
-        <v>76.094132</v>
+        <v>85.22542799999999</v>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
@@ -3135,7 +3135,7 @@
         <v>1.015102</v>
       </c>
       <c r="D36" s="0" t="n">
-        <v>215.404921</v>
+        <v>241.253512</v>
       </c>
       <c r="E36" s="0" t="inlineStr">
         <is>
@@ -3189,7 +3189,7 @@
         <v>0.8120810000000001</v>
       </c>
       <c r="D37" s="0" t="n">
-        <v>398.030833</v>
+        <v>445.794533</v>
       </c>
       <c r="E37" s="0" t="inlineStr">
         <is>
@@ -3297,7 +3297,7 @@
         <v>1.118287</v>
       </c>
       <c r="D39" s="0" t="n">
-        <v>112.415258</v>
+        <v>125.905089</v>
       </c>
       <c r="E39" s="0" t="inlineStr">
         <is>
@@ -3351,7 +3351,7 @@
         <v>1.067456</v>
       </c>
       <c r="D40" s="0" t="n">
-        <v>73.069918</v>
+        <v>81.838308</v>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
@@ -3405,7 +3405,7 @@
         <v>1.016624</v>
       </c>
       <c r="D41" s="0" t="n">
-        <v>206.844081</v>
+        <v>231.665371</v>
       </c>
       <c r="E41" s="0" t="inlineStr">
         <is>
@@ -3459,7 +3459,7 @@
         <v>0.813299</v>
       </c>
       <c r="D42" s="0" t="n">
-        <v>382.211883</v>
+        <v>428.077309</v>
       </c>
       <c r="E42" s="0" t="inlineStr">
         <is>
@@ -3567,7 +3567,7 @@
         <v>1.119964</v>
       </c>
       <c r="D44" s="0" t="n">
-        <v>128.947725</v>
+        <v>144.421452</v>
       </c>
       <c r="E44" s="0" t="inlineStr">
         <is>
@@ -3621,7 +3621,7 @@
         <v>1.069057</v>
       </c>
       <c r="D45" s="0" t="n">
-        <v>83.816022</v>
+        <v>93.87394500000001</v>
       </c>
       <c r="E45" s="0" t="inlineStr">
         <is>
@@ -3675,7 +3675,7 @@
         <v>1.018149</v>
       </c>
       <c r="D46" s="0" t="n">
-        <v>237.263818</v>
+        <v>265.735476</v>
       </c>
       <c r="E46" s="0" t="inlineStr">
         <is>
@@ -3729,7 +3729,7 @@
         <v>0.814519</v>
       </c>
       <c r="D47" s="0" t="n">
-        <v>438.422268</v>
+        <v>491.03294</v>
       </c>
       <c r="E47" s="0" t="inlineStr">
         <is>
@@ -3837,7 +3837,7 @@
         <v>1.121644</v>
       </c>
       <c r="D49" s="0" t="n">
-        <v>148.638422</v>
+        <v>166.475033</v>
       </c>
       <c r="E49" s="0" t="inlineStr">
         <is>
@@ -3891,7 +3891,7 @@
         <v>1.07066</v>
       </c>
       <c r="D50" s="0" t="n">
-        <v>96.614977</v>
+        <v>108.208774</v>
       </c>
       <c r="E50" s="0" t="inlineStr">
         <is>
@@ -3945,7 +3945,7 @@
         <v>1.019676</v>
       </c>
       <c r="D51" s="0" t="n">
-        <v>273.494699</v>
+        <v>306.314063</v>
       </c>
       <c r="E51" s="0" t="inlineStr">
         <is>
@@ -3999,7 +3999,7 @@
         <v>0.815741</v>
       </c>
       <c r="D52" s="0" t="n">
-        <v>505.370639</v>
+        <v>566.015116</v>
       </c>
       <c r="E52" s="0" t="inlineStr">
         <is>
@@ -4377,7 +4377,7 @@
         <v>1.125012</v>
       </c>
       <c r="D59" s="0" t="n">
-        <v>204.099421</v>
+        <v>228.591352</v>
       </c>
       <c r="E59" s="0" t="inlineStr">
         <is>
@@ -4431,7 +4431,7 @@
         <v>1.073875</v>
       </c>
       <c r="D60" s="0" t="n">
-        <v>132.664624</v>
+        <v>148.584379</v>
       </c>
       <c r="E60" s="0" t="inlineStr">
         <is>
@@ -4485,7 +4485,7 @@
         <v>1.022738</v>
       </c>
       <c r="D61" s="0" t="n">
-        <v>375.542936</v>
+        <v>420.608088</v>
       </c>
       <c r="E61" s="0" t="inlineStr">
         <is>
@@ -4539,7 +4539,7 @@
         <v>0.81819</v>
       </c>
       <c r="D62" s="0" t="n">
-        <v>693.938036</v>
+        <v>777.2106</v>
       </c>
       <c r="E62" s="0" t="inlineStr">
         <is>
@@ -4647,7 +4647,7 @@
         <v>1.126699</v>
       </c>
       <c r="D64" s="0" t="n">
-        <v>196.470027</v>
+        <v>220.04643</v>
       </c>
       <c r="E64" s="0" t="inlineStr">
         <is>
@@ -4701,7 +4701,7 @@
         <v>1.075485</v>
       </c>
       <c r="D65" s="0" t="n">
-        <v>127.705517</v>
+        <v>143.030179</v>
       </c>
       <c r="E65" s="0" t="inlineStr">
         <is>
@@ -4755,7 +4755,7 @@
         <v>1.024272</v>
       </c>
       <c r="D66" s="0" t="n">
-        <v>361.50485</v>
+        <v>404.885432</v>
       </c>
       <c r="E66" s="0" t="inlineStr">
         <is>
@@ -4809,7 +4809,7 @@
         <v>0.819418</v>
       </c>
       <c r="D67" s="0" t="n">
-        <v>667.998094</v>
+        <v>748.157865</v>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
@@ -4917,7 +4917,7 @@
         <v>1.128389</v>
       </c>
       <c r="D69" s="0" t="n">
-        <v>199.998048</v>
+        <v>223.997814</v>
       </c>
       <c r="E69" s="0" t="inlineStr">
         <is>
@@ -4971,7 +4971,7 @@
         <v>1.077099</v>
       </c>
       <c r="D70" s="0" t="n">
-        <v>129.998731</v>
+        <v>145.598579</v>
       </c>
       <c r="E70" s="0" t="inlineStr">
         <is>
@@ -5025,7 +5025,7 @@
         <v>1.025808</v>
       </c>
       <c r="D71" s="0" t="n">
-        <v>367.996407</v>
+        <v>412.155976</v>
       </c>
       <c r="E71" s="0" t="inlineStr">
         <is>
@@ -5079,7 +5079,7 @@
         <v>0.820647</v>
       </c>
       <c r="D72" s="0" t="n">
-        <v>679.993363</v>
+        <v>761.592567</v>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
@@ -5187,7 +5187,7 @@
         <v>1.130082</v>
       </c>
       <c r="D74" s="0" t="n">
-        <v>223.81389</v>
+        <v>250.671557</v>
       </c>
       <c r="E74" s="0" t="inlineStr">
         <is>
@@ -5241,7 +5241,7 @@
         <v>1.078714</v>
       </c>
       <c r="D75" s="0" t="n">
-        <v>145.479031</v>
+        <v>162.936515</v>
       </c>
       <c r="E75" s="0" t="inlineStr">
         <is>
@@ -5295,7 +5295,7 @@
         <v>1.027347</v>
       </c>
       <c r="D76" s="0" t="n">
-        <v>411.817556</v>
+        <v>461.235663</v>
       </c>
       <c r="E76" s="0" t="inlineStr">
         <is>
@@ -5349,7 +5349,7 @@
         <v>0.821878</v>
       </c>
       <c r="D77" s="0" t="n">
-        <v>760.967224</v>
+        <v>852.283291</v>
       </c>
       <c r="E77" s="0" t="inlineStr">
         <is>
@@ -5727,7 +5727,7 @@
         <v>1.133475</v>
       </c>
       <c r="D84" s="0" t="n">
-        <v>352.658185</v>
+        <v>394.977167</v>
       </c>
       <c r="E84" s="0" t="inlineStr">
         <is>
@@ -5781,7 +5781,7 @@
         <v>1.081953</v>
       </c>
       <c r="D85" s="0" t="n">
-        <v>229.227821</v>
+        <v>256.73516</v>
       </c>
       <c r="E85" s="0" t="inlineStr">
         <is>
@@ -5835,7 +5835,7 @@
         <v>1.030431</v>
       </c>
       <c r="D86" s="0" t="n">
-        <v>648.891062</v>
+        <v>726.757989</v>
       </c>
       <c r="E86" s="0" t="inlineStr">
         <is>
@@ -5889,7 +5889,7 @@
         <v>0.824345</v>
       </c>
       <c r="D87" s="0" t="n">
-        <v>1199.037828</v>
+        <v>1342.922367</v>
       </c>
       <c r="E87" s="0" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v>1.135175</v>
       </c>
       <c r="D89" s="0" t="n">
-        <v>344.100103</v>
+        <v>385.392115</v>
       </c>
       <c r="E89" s="0" t="inlineStr">
         <is>
@@ -6051,7 +6051,7 @@
         <v>1.083576</v>
       </c>
       <c r="D90" s="0" t="n">
-        <v>223.665066</v>
+        <v>250.504874</v>
       </c>
       <c r="E90" s="0" t="inlineStr">
         <is>
@@ -6105,7 +6105,7 @@
         <v>1.031977</v>
       </c>
       <c r="D91" s="0" t="n">
-        <v>633.144186</v>
+        <v>709.121488</v>
       </c>
       <c r="E91" s="0" t="inlineStr">
         <is>
@@ -6159,7 +6159,7 @@
         <v>0.825582</v>
       </c>
       <c r="D92" s="0" t="n">
-        <v>1169.940346</v>
+        <v>1310.333188</v>
       </c>
       <c r="E92" s="0" t="inlineStr">
         <is>
@@ -6267,7 +6267,7 @@
         <v>1.136877</v>
       </c>
       <c r="D94" s="0" t="n">
-        <v>337.333158</v>
+        <v>377.813137</v>
       </c>
       <c r="E94" s="0" t="inlineStr">
         <is>
@@ -6321,7 +6321,7 @@
         <v>1.085201</v>
       </c>
       <c r="D95" s="0" t="n">
-        <v>219.266552</v>
+        <v>245.578538</v>
       </c>
       <c r="E95" s="0" t="inlineStr">
         <is>
@@ -6375,7 +6375,7 @@
         <v>1.033525</v>
       </c>
       <c r="D96" s="0" t="n">
-        <v>620.6930139999999</v>
+        <v>695.1761760000001</v>
       </c>
       <c r="E96" s="0" t="inlineStr">
         <is>
@@ -6429,7 +6429,7 @@
         <v>0.82682</v>
       </c>
       <c r="D97" s="0" t="n">
-        <v>1146.932738</v>
+        <v>1284.564667</v>
       </c>
       <c r="E97" s="0" t="inlineStr">
         <is>
@@ -6537,7 +6537,7 @@
         <v>1.138583</v>
       </c>
       <c r="D99" s="0" t="n">
-        <v>350.500216</v>
+        <v>392.560242</v>
       </c>
       <c r="E99" s="0" t="inlineStr">
         <is>
@@ -6591,7 +6591,7 @@
         <v>1.086829</v>
       </c>
       <c r="D100" s="0" t="n">
-        <v>227.825143</v>
+        <v>255.16416</v>
       </c>
       <c r="E100" s="0" t="inlineStr">
         <is>
@@ -6645,7 +6645,7 @@
         <v>1.035075</v>
       </c>
       <c r="D101" s="0" t="n">
-        <v>644.920401</v>
+        <v>722.310849</v>
       </c>
       <c r="E101" s="0" t="inlineStr">
         <is>
@@ -6699,7 +6699,7 @@
         <v>0.82806</v>
       </c>
       <c r="D102" s="0" t="n">
-        <v>1191.70074</v>
+        <v>1334.704829</v>
       </c>
       <c r="E102" s="0" t="inlineStr">
         <is>
@@ -6807,7 +6807,7 @@
         <v>1.140291</v>
       </c>
       <c r="D104" s="0" t="n">
-        <v>458.698495</v>
+        <v>435.76357</v>
       </c>
       <c r="E104" s="0" t="inlineStr">
         <is>
@@ -6861,7 +6861,7 @@
         <v>1.088459</v>
       </c>
       <c r="D105" s="0" t="n">
-        <v>298.154022</v>
+        <v>283.246321</v>
       </c>
       <c r="E105" s="0" t="inlineStr">
         <is>
@@ -6915,7 +6915,7 @@
         <v>1.036628</v>
       </c>
       <c r="D106" s="0" t="n">
-        <v>844.005229</v>
+        <v>801.804968</v>
       </c>
       <c r="E106" s="0" t="inlineStr">
         <is>
@@ -6969,7 +6969,7 @@
         <v>0.829302</v>
       </c>
       <c r="D107" s="0" t="n">
-        <v>1559.57488</v>
+        <v>1481.596136</v>
       </c>
       <c r="E107" s="0" t="inlineStr">
         <is>
@@ -7023,7 +7023,7 @@
         <v>0.777471</v>
       </c>
       <c r="D108" s="0" t="n">
-        <v>2504.493782</v>
+        <v>2379.269093</v>
       </c>
       <c r="E108" s="0" t="inlineStr">
         <is>
@@ -7077,7 +7077,7 @@
         <v>1.036628</v>
       </c>
       <c r="D109" s="0" t="n">
-        <v>766.192472</v>
+        <v>789.1782459999999</v>
       </c>
       <c r="E109" s="0" t="inlineStr">
         <is>

</xml_diff>